<commit_message>
feat: implement ML pipeline hyperparameter tuning, 80/20 train/test splits, dynamic metrics, and Fast2SMS reminder gateway
</commit_message>
<xml_diff>
--- a/datasets/schemes_dataset.xlsx
+++ b/datasets/schemes_dataset.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,11 +514,7 @@
       <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -674,11 +670,7 @@
       <c r="I6" t="n">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -714,11 +706,7 @@
       <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -834,11 +822,7 @@
       <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -994,11 +978,7 @@
       <c r="I14" t="n">
         <v>0</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1194,11 +1174,7 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1234,11 +1210,7 @@
       <c r="I20" t="n">
         <v>0</v>
       </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1634,11 +1606,7 @@
       <c r="I30" t="n">
         <v>0</v>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1674,11 +1642,7 @@
       <c r="I31" t="n">
         <v>0</v>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1994,11 +1958,7 @@
       <c r="I39" t="n">
         <v>0</v>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2354,11 +2314,7 @@
       <c r="I48" t="n">
         <v>0</v>
       </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2754,11 +2710,7 @@
       <c r="I58" t="n">
         <v>0</v>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2874,11 +2826,7 @@
       <c r="I61" t="n">
         <v>0</v>
       </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2914,11 +2862,7 @@
       <c r="I62" t="n">
         <v>0</v>
       </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3074,11 +3018,7 @@
       <c r="I66" t="n">
         <v>0</v>
       </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3194,11 +3134,7 @@
       <c r="I69" t="n">
         <v>1</v>
       </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3514,11 +3450,7 @@
       <c r="I77" t="n">
         <v>0</v>
       </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3874,11 +3806,7 @@
       <c r="I86" t="n">
         <v>0</v>
       </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4034,11 +3962,7 @@
       <c r="I90" t="n">
         <v>1</v>
       </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4234,11 +4158,7 @@
       <c r="I95" t="n">
         <v>0</v>
       </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4274,11 +4194,7 @@
       <c r="I96" t="n">
         <v>0</v>
       </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5034,11 +4950,7 @@
       <c r="I115" t="n">
         <v>0</v>
       </c>
-      <c r="J115" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5354,11 +5266,7 @@
       <c r="I123" t="n">
         <v>0</v>
       </c>
-      <c r="J123" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5434,11 +5342,7 @@
       <c r="I125" t="n">
         <v>0</v>
       </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6154,11 +6058,7 @@
       <c r="I143" t="n">
         <v>0</v>
       </c>
-      <c r="J143" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6234,11 +6134,7 @@
       <c r="I145" t="n">
         <v>0</v>
       </c>
-      <c r="J145" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6554,11 +6450,7 @@
       <c r="I153" t="n">
         <v>0</v>
       </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
+      <c r="J153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6883,11 +6775,11 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>S_SEED_161</t>
+          <t>S_DB_1</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
@@ -6896,42 +6788,42 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>64501.39</v>
+        <v>75000</v>
       </c>
       <c r="F162" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G162" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H162" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I162" t="n">
         <v>0</v>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>Post-Matric Scholarship</t>
+          <t>PM Kisan</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>S_SEED_162</t>
+          <t>S_DB_2</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -6940,13 +6832,13 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>282474.01</v>
+        <v>48000</v>
       </c>
       <c r="F163" t="n">
-        <v>3.17</v>
+        <v>0.2</v>
       </c>
       <c r="G163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H163" t="n">
         <v>0</v>
@@ -6956,58 +6848,58 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>MGNREGA</t>
+          <t>PM Awas Yojana</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>S_SEED_163</t>
+          <t>S_DB_3</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>33408.75</v>
+        <v>240000</v>
       </c>
       <c r="F164" t="n">
-        <v>2.1</v>
+        <v>1.2</v>
       </c>
       <c r="G164" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H164" t="n">
         <v>0</v>
       </c>
       <c r="I164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>PM Kisan</t>
+          <t>None</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>S_SEED_164</t>
+          <t>S_DB_4</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
@@ -7016,38 +6908,38 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Student</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>86509.02</v>
+        <v>35000</v>
       </c>
       <c r="F165" t="n">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="G165" t="n">
         <v>0</v>
       </c>
       <c r="H165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I165" t="n">
         <v>0</v>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>PM Awas Yojana</t>
+          <t>Post-Matric Scholarship</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>S_SEED_165</t>
+          <t>S_DB_5</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
@@ -7056,17 +6948,17 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>316013.03</v>
+        <v>145000</v>
       </c>
       <c r="F166" t="n">
-        <v>3.48</v>
+        <v>0.5</v>
       </c>
       <c r="G166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H166" t="n">
         <v>0</v>
@@ -7076,1407 +6968,7 @@
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>S_SEED_166</t>
-        </is>
-      </c>
-      <c r="B167" t="n">
-        <v>56</v>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E167" t="n">
-        <v>436110.74</v>
-      </c>
-      <c r="F167" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="G167" t="n">
-        <v>1</v>
-      </c>
-      <c r="H167" t="n">
-        <v>0</v>
-      </c>
-      <c r="I167" t="n">
-        <v>0</v>
-      </c>
-      <c r="J167" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>S_SEED_167</t>
-        </is>
-      </c>
-      <c r="B168" t="n">
-        <v>29</v>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>Unemployed</t>
-        </is>
-      </c>
-      <c r="E168" t="n">
-        <v>78832.00999999999</v>
-      </c>
-      <c r="F168" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="G168" t="n">
-        <v>1</v>
-      </c>
-      <c r="H168" t="n">
-        <v>0</v>
-      </c>
-      <c r="I168" t="n">
-        <v>0</v>
-      </c>
-      <c r="J168" t="inlineStr">
-        <is>
-          <t>MGNREGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>S_SEED_168</t>
-        </is>
-      </c>
-      <c r="B169" t="n">
-        <v>64</v>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="E169" t="n">
-        <v>294748.24</v>
-      </c>
-      <c r="F169" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="G169" t="n">
-        <v>0</v>
-      </c>
-      <c r="H169" t="n">
-        <v>0</v>
-      </c>
-      <c r="I169" t="n">
-        <v>1</v>
-      </c>
-      <c r="J169" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>S_SEED_169</t>
-        </is>
-      </c>
-      <c r="B170" t="n">
-        <v>33</v>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E170" t="n">
-        <v>115120.06</v>
-      </c>
-      <c r="F170" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="G170" t="n">
-        <v>1</v>
-      </c>
-      <c r="H170" t="n">
-        <v>0</v>
-      </c>
-      <c r="I170" t="n">
-        <v>0</v>
-      </c>
-      <c r="J170" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>S_SEED_170</t>
-        </is>
-      </c>
-      <c r="B171" t="n">
-        <v>62</v>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>Laborer</t>
-        </is>
-      </c>
-      <c r="E171" t="n">
-        <v>449722</v>
-      </c>
-      <c r="F171" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="G171" t="n">
-        <v>0</v>
-      </c>
-      <c r="H171" t="n">
-        <v>0</v>
-      </c>
-      <c r="I171" t="n">
-        <v>0</v>
-      </c>
-      <c r="J171" t="inlineStr">
-        <is>
-          <t>MGNREGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>S_SEED_171</t>
-        </is>
-      </c>
-      <c r="B172" t="n">
-        <v>24</v>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E172" t="n">
-        <v>417490.36</v>
-      </c>
-      <c r="F172" t="n">
-        <v>7.77</v>
-      </c>
-      <c r="G172" t="n">
-        <v>1</v>
-      </c>
-      <c r="H172" t="n">
-        <v>0</v>
-      </c>
-      <c r="I172" t="n">
-        <v>0</v>
-      </c>
-      <c r="J172" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>S_SEED_172</t>
-        </is>
-      </c>
-      <c r="B173" t="n">
-        <v>40</v>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E173" t="n">
-        <v>215711.78</v>
-      </c>
-      <c r="F173" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="G173" t="n">
-        <v>1</v>
-      </c>
-      <c r="H173" t="n">
-        <v>0</v>
-      </c>
-      <c r="I173" t="n">
-        <v>0</v>
-      </c>
-      <c r="J173" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>S_SEED_173</t>
-        </is>
-      </c>
-      <c r="B174" t="n">
-        <v>56</v>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E174" t="n">
-        <v>71843.75999999999</v>
-      </c>
-      <c r="F174" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="G174" t="n">
-        <v>1</v>
-      </c>
-      <c r="H174" t="n">
-        <v>0</v>
-      </c>
-      <c r="I174" t="n">
-        <v>0</v>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>S_SEED_174</t>
-        </is>
-      </c>
-      <c r="B175" t="n">
-        <v>54</v>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E175" t="n">
-        <v>266143.94</v>
-      </c>
-      <c r="F175" t="n">
-        <v>6.43</v>
-      </c>
-      <c r="G175" t="n">
-        <v>1</v>
-      </c>
-      <c r="H175" t="n">
-        <v>0</v>
-      </c>
-      <c r="I175" t="n">
-        <v>0</v>
-      </c>
-      <c r="J175" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>S_SEED_175</t>
-        </is>
-      </c>
-      <c r="B176" t="n">
-        <v>21</v>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="E176" t="n">
-        <v>284821.17</v>
-      </c>
-      <c r="F176" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G176" t="n">
-        <v>0</v>
-      </c>
-      <c r="H176" t="n">
-        <v>0</v>
-      </c>
-      <c r="I176" t="n">
-        <v>0</v>
-      </c>
-      <c r="J176" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>S_SEED_176</t>
-        </is>
-      </c>
-      <c r="B177" t="n">
-        <v>59</v>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E177" t="n">
-        <v>185104.47</v>
-      </c>
-      <c r="F177" t="n">
-        <v>7.46</v>
-      </c>
-      <c r="G177" t="n">
-        <v>1</v>
-      </c>
-      <c r="H177" t="n">
-        <v>0</v>
-      </c>
-      <c r="I177" t="n">
-        <v>0</v>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>S_SEED_177</t>
-        </is>
-      </c>
-      <c r="B178" t="n">
-        <v>56</v>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E178" t="n">
-        <v>36166.61</v>
-      </c>
-      <c r="F178" t="n">
-        <v>3.84</v>
-      </c>
-      <c r="G178" t="n">
-        <v>1</v>
-      </c>
-      <c r="H178" t="n">
-        <v>0</v>
-      </c>
-      <c r="I178" t="n">
-        <v>0</v>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>S_SEED_178</t>
-        </is>
-      </c>
-      <c r="B179" t="n">
-        <v>33</v>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="E179" t="n">
-        <v>199639.72</v>
-      </c>
-      <c r="F179" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="G179" t="n">
-        <v>0</v>
-      </c>
-      <c r="H179" t="n">
-        <v>0</v>
-      </c>
-      <c r="I179" t="n">
-        <v>1</v>
-      </c>
-      <c r="J179" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>S_SEED_179</t>
-        </is>
-      </c>
-      <c r="B180" t="n">
-        <v>47</v>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E180" t="n">
-        <v>386713.38</v>
-      </c>
-      <c r="F180" t="n">
-        <v>5.72</v>
-      </c>
-      <c r="G180" t="n">
-        <v>1</v>
-      </c>
-      <c r="H180" t="n">
-        <v>0</v>
-      </c>
-      <c r="I180" t="n">
-        <v>0</v>
-      </c>
-      <c r="J180" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>S_SEED_180</t>
-        </is>
-      </c>
-      <c r="B181" t="n">
-        <v>54</v>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E181" t="n">
-        <v>203942.45</v>
-      </c>
-      <c r="F181" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="G181" t="n">
-        <v>0</v>
-      </c>
-      <c r="H181" t="n">
-        <v>0</v>
-      </c>
-      <c r="I181" t="n">
-        <v>0</v>
-      </c>
-      <c r="J181" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>S_SEED_181</t>
-        </is>
-      </c>
-      <c r="B182" t="n">
-        <v>29</v>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E182" t="n">
-        <v>273078.32</v>
-      </c>
-      <c r="F182" t="n">
-        <v>7.86</v>
-      </c>
-      <c r="G182" t="n">
-        <v>1</v>
-      </c>
-      <c r="H182" t="n">
-        <v>0</v>
-      </c>
-      <c r="I182" t="n">
-        <v>0</v>
-      </c>
-      <c r="J182" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>S_SEED_182</t>
-        </is>
-      </c>
-      <c r="B183" t="n">
-        <v>63</v>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E183" t="n">
-        <v>339641.71</v>
-      </c>
-      <c r="F183" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G183" t="n">
-        <v>0</v>
-      </c>
-      <c r="H183" t="n">
-        <v>0</v>
-      </c>
-      <c r="I183" t="n">
-        <v>0</v>
-      </c>
-      <c r="J183" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>S_SEED_183</t>
-        </is>
-      </c>
-      <c r="B184" t="n">
-        <v>46</v>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>Laborer</t>
-        </is>
-      </c>
-      <c r="E184" t="n">
-        <v>119188.02</v>
-      </c>
-      <c r="F184" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="G184" t="n">
-        <v>0</v>
-      </c>
-      <c r="H184" t="n">
-        <v>0</v>
-      </c>
-      <c r="I184" t="n">
-        <v>0</v>
-      </c>
-      <c r="J184" t="inlineStr">
-        <is>
-          <t>PM Awas Yojana</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>S_SEED_184</t>
-        </is>
-      </c>
-      <c r="B185" t="n">
-        <v>66</v>
-      </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="E185" t="n">
-        <v>290804.51</v>
-      </c>
-      <c r="F185" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="G185" t="n">
-        <v>0</v>
-      </c>
-      <c r="H185" t="n">
-        <v>0</v>
-      </c>
-      <c r="I185" t="n">
-        <v>0</v>
-      </c>
-      <c r="J185" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>S_SEED_185</t>
-        </is>
-      </c>
-      <c r="B186" t="n">
-        <v>37</v>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E186" t="n">
-        <v>346042.54</v>
-      </c>
-      <c r="F186" t="n">
-        <v>5.57</v>
-      </c>
-      <c r="G186" t="n">
-        <v>1</v>
-      </c>
-      <c r="H186" t="n">
-        <v>0</v>
-      </c>
-      <c r="I186" t="n">
-        <v>0</v>
-      </c>
-      <c r="J186" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>S_SEED_186</t>
-        </is>
-      </c>
-      <c r="B187" t="n">
-        <v>41</v>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>Laborer</t>
-        </is>
-      </c>
-      <c r="E187" t="n">
-        <v>341584.79</v>
-      </c>
-      <c r="F187" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="G187" t="n">
-        <v>0</v>
-      </c>
-      <c r="H187" t="n">
-        <v>0</v>
-      </c>
-      <c r="I187" t="n">
-        <v>0</v>
-      </c>
-      <c r="J187" t="inlineStr">
-        <is>
-          <t>MGNREGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>S_SEED_187</t>
-        </is>
-      </c>
-      <c r="B188" t="n">
-        <v>54</v>
-      </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E188" t="n">
-        <v>75691.42</v>
-      </c>
-      <c r="F188" t="n">
-        <v>7.11</v>
-      </c>
-      <c r="G188" t="n">
-        <v>1</v>
-      </c>
-      <c r="H188" t="n">
-        <v>0</v>
-      </c>
-      <c r="I188" t="n">
-        <v>0</v>
-      </c>
-      <c r="J188" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>S_SEED_188</t>
-        </is>
-      </c>
-      <c r="B189" t="n">
-        <v>42</v>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E189" t="n">
-        <v>420583.48</v>
-      </c>
-      <c r="F189" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="G189" t="n">
-        <v>1</v>
-      </c>
-      <c r="H189" t="n">
-        <v>0</v>
-      </c>
-      <c r="I189" t="n">
-        <v>0</v>
-      </c>
-      <c r="J189" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>S_SEED_189</t>
-        </is>
-      </c>
-      <c r="B190" t="n">
-        <v>51</v>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E190" t="n">
-        <v>331070.65</v>
-      </c>
-      <c r="F190" t="n">
-        <v>3.97</v>
-      </c>
-      <c r="G190" t="n">
-        <v>1</v>
-      </c>
-      <c r="H190" t="n">
-        <v>0</v>
-      </c>
-      <c r="I190" t="n">
-        <v>0</v>
-      </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>S_SEED_190</t>
-        </is>
-      </c>
-      <c r="B191" t="n">
-        <v>23</v>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E191" t="n">
-        <v>46452.32</v>
-      </c>
-      <c r="F191" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="G191" t="n">
-        <v>1</v>
-      </c>
-      <c r="H191" t="n">
-        <v>0</v>
-      </c>
-      <c r="I191" t="n">
-        <v>0</v>
-      </c>
-      <c r="J191" t="inlineStr">
-        <is>
-          <t>MGNREGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>S_SEED_191</t>
-        </is>
-      </c>
-      <c r="B192" t="n">
-        <v>68</v>
-      </c>
-      <c r="C192" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>Laborer</t>
-        </is>
-      </c>
-      <c r="E192" t="n">
-        <v>263264.74</v>
-      </c>
-      <c r="F192" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="G192" t="n">
-        <v>0</v>
-      </c>
-      <c r="H192" t="n">
-        <v>0</v>
-      </c>
-      <c r="I192" t="n">
-        <v>0</v>
-      </c>
-      <c r="J192" t="inlineStr">
-        <is>
-          <t>MGNREGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>S_SEED_192</t>
-        </is>
-      </c>
-      <c r="B193" t="n">
-        <v>36</v>
-      </c>
-      <c r="C193" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E193" t="n">
-        <v>88972.05</v>
-      </c>
-      <c r="F193" t="n">
-        <v>2.67</v>
-      </c>
-      <c r="G193" t="n">
-        <v>1</v>
-      </c>
-      <c r="H193" t="n">
-        <v>0</v>
-      </c>
-      <c r="I193" t="n">
-        <v>0</v>
-      </c>
-      <c r="J193" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>S_SEED_193</t>
-        </is>
-      </c>
-      <c r="B194" t="n">
-        <v>62</v>
-      </c>
-      <c r="C194" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>Laborer</t>
-        </is>
-      </c>
-      <c r="E194" t="n">
-        <v>343668.16</v>
-      </c>
-      <c r="F194" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="G194" t="n">
-        <v>0</v>
-      </c>
-      <c r="H194" t="n">
-        <v>0</v>
-      </c>
-      <c r="I194" t="n">
-        <v>0</v>
-      </c>
-      <c r="J194" t="inlineStr">
-        <is>
-          <t>MGNREGA</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>S_SEED_194</t>
-        </is>
-      </c>
-      <c r="B195" t="n">
-        <v>74</v>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E195" t="n">
-        <v>164101.11</v>
-      </c>
-      <c r="F195" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="G195" t="n">
-        <v>1</v>
-      </c>
-      <c r="H195" t="n">
-        <v>0</v>
-      </c>
-      <c r="I195" t="n">
-        <v>0</v>
-      </c>
-      <c r="J195" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>S_SEED_195</t>
-        </is>
-      </c>
-      <c r="B196" t="n">
-        <v>48</v>
-      </c>
-      <c r="C196" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="E196" t="n">
-        <v>131235.98</v>
-      </c>
-      <c r="F196" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="G196" t="n">
-        <v>0</v>
-      </c>
-      <c r="H196" t="n">
-        <v>0</v>
-      </c>
-      <c r="I196" t="n">
-        <v>0</v>
-      </c>
-      <c r="J196" t="inlineStr">
-        <is>
-          <t>PM Awas Yojana</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>S_SEED_196</t>
-        </is>
-      </c>
-      <c r="B197" t="n">
-        <v>44</v>
-      </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E197" t="n">
-        <v>292622.45</v>
-      </c>
-      <c r="F197" t="n">
-        <v>4.32</v>
-      </c>
-      <c r="G197" t="n">
-        <v>1</v>
-      </c>
-      <c r="H197" t="n">
-        <v>0</v>
-      </c>
-      <c r="I197" t="n">
-        <v>0</v>
-      </c>
-      <c r="J197" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>S_SEED_197</t>
-        </is>
-      </c>
-      <c r="B198" t="n">
-        <v>52</v>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E198" t="n">
-        <v>205863.54</v>
-      </c>
-      <c r="F198" t="n">
-        <v>6.72</v>
-      </c>
-      <c r="G198" t="n">
-        <v>1</v>
-      </c>
-      <c r="H198" t="n">
-        <v>0</v>
-      </c>
-      <c r="I198" t="n">
-        <v>0</v>
-      </c>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>S_SEED_198</t>
-        </is>
-      </c>
-      <c r="B199" t="n">
-        <v>45</v>
-      </c>
-      <c r="C199" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>Agriculture</t>
-        </is>
-      </c>
-      <c r="E199" t="n">
-        <v>423008.25</v>
-      </c>
-      <c r="F199" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G199" t="n">
-        <v>1</v>
-      </c>
-      <c r="H199" t="n">
-        <v>0</v>
-      </c>
-      <c r="I199" t="n">
-        <v>1</v>
-      </c>
-      <c r="J199" t="inlineStr">
-        <is>
-          <t>PM Kisan</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>S_SEED_199</t>
-        </is>
-      </c>
-      <c r="B200" t="n">
-        <v>67</v>
-      </c>
-      <c r="C200" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>Business</t>
-        </is>
-      </c>
-      <c r="E200" t="n">
-        <v>324685.96</v>
-      </c>
-      <c r="F200" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="G200" t="n">
-        <v>0</v>
-      </c>
-      <c r="H200" t="n">
-        <v>0</v>
-      </c>
-      <c r="I200" t="n">
-        <v>0</v>
-      </c>
-      <c r="J200" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>S_SEED_200</t>
-        </is>
-      </c>
-      <c r="B201" t="n">
-        <v>73</v>
-      </c>
-      <c r="C201" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E201" t="n">
-        <v>436617.48</v>
-      </c>
-      <c r="F201" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="G201" t="n">
-        <v>0</v>
-      </c>
-      <c r="H201" t="n">
-        <v>0</v>
-      </c>
-      <c r="I201" t="n">
-        <v>0</v>
-      </c>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t>No Scheme</t>
+          <t>None</t>
         </is>
       </c>
     </row>

</xml_diff>